<commit_message>
Add students data for deployment
</commit_message>
<xml_diff>
--- a/votes.xlsx
+++ b/votes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study-Materials\SUST\Election\server\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54664FE0-8716-4F4D-9735-4E4911D44B94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAD8BED8-6962-484F-A95E-CFE9B4E28FB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,18 +20,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
     <t>Candidate</t>
   </si>
   <si>
     <t>Time</t>
-  </si>
-  <si>
-    <t>Candidate A</t>
-  </si>
-  <si>
-    <t>2026-07-28T22:06:14.402Z</t>
   </si>
 </sst>
 </file>
@@ -408,13 +402,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.5"/>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="22.8125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -422,18 +416,10 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:B2" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:B1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>